<commit_message>
Sheets: CC's full unit-economics stack (warehousing, payout 6%+$0.30 = 7% fee share, refunds, creators+ads; reproduces $29.99 -> 31.92/38.92/56.08/26.08%/54.76 in Python, JS and browser engines + xlsx), ad stop-loss line, new Scale Ceiling sheet, three-batch cash check, market stage = CC's 3 stages with example markets (stage 4 labelled aiOS addition) + supply-chain gate + routes by background, 6-second/60% hook gate, one selling point per week, aiOS-default labels; tests
</commit_message>
<xml_diff>
--- a/templates/xlsx/asset-log.xlsx
+++ b/templates/xlsx/asset-log.xlsx
@@ -508,7 +508,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>3s retention %</t>
+          <t>6s retention % (gate ≈60%)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -596,7 +596,7 @@
         <v/>
       </c>
       <c r="M2" s="6">
-        <f>IF(A2="","",IF(F2=0,"",IF(G2&lt;0.25,"P0 fix hook",IF(AND(D2="Harvest",I2=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A2="","",IF(F2=0,"",IF(G2&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D2="Harvest",I2=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -610,7 +610,7 @@
         <v/>
       </c>
       <c r="M3" s="6">
-        <f>IF(A3="","",IF(F3=0,"",IF(G3&lt;0.25,"P0 fix hook",IF(AND(D3="Harvest",I3=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A3="","",IF(F3=0,"",IF(G3&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D3="Harvest",I3=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -624,7 +624,7 @@
         <v/>
       </c>
       <c r="M4" s="6">
-        <f>IF(A4="","",IF(F4=0,"",IF(G4&lt;0.25,"P0 fix hook",IF(AND(D4="Harvest",I4=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A4="","",IF(F4=0,"",IF(G4&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D4="Harvest",I4=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -638,7 +638,7 @@
         <v/>
       </c>
       <c r="M5" s="6">
-        <f>IF(A5="","",IF(F5=0,"",IF(G5&lt;0.25,"P0 fix hook",IF(AND(D5="Harvest",I5=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A5="","",IF(F5=0,"",IF(G5&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D5="Harvest",I5=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -652,7 +652,7 @@
         <v/>
       </c>
       <c r="M6" s="6">
-        <f>IF(A6="","",IF(F6=0,"",IF(G6&lt;0.25,"P0 fix hook",IF(AND(D6="Harvest",I6=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A6="","",IF(F6=0,"",IF(G6&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D6="Harvest",I6=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -666,7 +666,7 @@
         <v/>
       </c>
       <c r="M7" s="6">
-        <f>IF(A7="","",IF(F7=0,"",IF(G7&lt;0.25,"P0 fix hook",IF(AND(D7="Harvest",I7=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A7="","",IF(F7=0,"",IF(G7&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D7="Harvest",I7=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -680,7 +680,7 @@
         <v/>
       </c>
       <c r="M8" s="6">
-        <f>IF(A8="","",IF(F8=0,"",IF(G8&lt;0.25,"P0 fix hook",IF(AND(D8="Harvest",I8=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A8="","",IF(F8=0,"",IF(G8&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D8="Harvest",I8=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -694,7 +694,7 @@
         <v/>
       </c>
       <c r="M9" s="6">
-        <f>IF(A9="","",IF(F9=0,"",IF(G9&lt;0.25,"P0 fix hook",IF(AND(D9="Harvest",I9=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A9="","",IF(F9=0,"",IF(G9&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D9="Harvest",I9=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -708,7 +708,7 @@
         <v/>
       </c>
       <c r="M10" s="6">
-        <f>IF(A10="","",IF(F10=0,"",IF(G10&lt;0.25,"P0 fix hook",IF(AND(D10="Harvest",I10=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A10="","",IF(F10=0,"",IF(G10&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D10="Harvest",I10=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -722,7 +722,7 @@
         <v/>
       </c>
       <c r="M11" s="6">
-        <f>IF(A11="","",IF(F11=0,"",IF(G11&lt;0.25,"P0 fix hook",IF(AND(D11="Harvest",I11=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A11="","",IF(F11=0,"",IF(G11&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D11="Harvest",I11=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -736,7 +736,7 @@
         <v/>
       </c>
       <c r="M12" s="6">
-        <f>IF(A12="","",IF(F12=0,"",IF(G12&lt;0.25,"P0 fix hook",IF(AND(D12="Harvest",I12=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A12="","",IF(F12=0,"",IF(G12&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D12="Harvest",I12=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -750,7 +750,7 @@
         <v/>
       </c>
       <c r="M13" s="6">
-        <f>IF(A13="","",IF(F13=0,"",IF(G13&lt;0.25,"P0 fix hook",IF(AND(D13="Harvest",I13=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A13="","",IF(F13=0,"",IF(G13&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D13="Harvest",I13=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -764,7 +764,7 @@
         <v/>
       </c>
       <c r="M14" s="6">
-        <f>IF(A14="","",IF(F14=0,"",IF(G14&lt;0.25,"P0 fix hook",IF(AND(D14="Harvest",I14=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A14="","",IF(F14=0,"",IF(G14&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D14="Harvest",I14=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -778,7 +778,7 @@
         <v/>
       </c>
       <c r="M15" s="6">
-        <f>IF(A15="","",IF(F15=0,"",IF(G15&lt;0.25,"P0 fix hook",IF(AND(D15="Harvest",I15=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A15="","",IF(F15=0,"",IF(G15&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D15="Harvest",I15=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -792,7 +792,7 @@
         <v/>
       </c>
       <c r="M16" s="6">
-        <f>IF(A16="","",IF(F16=0,"",IF(G16&lt;0.25,"P0 fix hook",IF(AND(D16="Harvest",I16=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A16="","",IF(F16=0,"",IF(G16&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D16="Harvest",I16=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -806,7 +806,7 @@
         <v/>
       </c>
       <c r="M17" s="6">
-        <f>IF(A17="","",IF(F17=0,"",IF(G17&lt;0.25,"P0 fix hook",IF(AND(D17="Harvest",I17=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A17="","",IF(F17=0,"",IF(G17&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D17="Harvest",I17=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -820,7 +820,7 @@
         <v/>
       </c>
       <c r="M18" s="6">
-        <f>IF(A18="","",IF(F18=0,"",IF(G18&lt;0.25,"P0 fix hook",IF(AND(D18="Harvest",I18=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A18="","",IF(F18=0,"",IF(G18&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D18="Harvest",I18=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -834,7 +834,7 @@
         <v/>
       </c>
       <c r="M19" s="6">
-        <f>IF(A19="","",IF(F19=0,"",IF(G19&lt;0.25,"P0 fix hook",IF(AND(D19="Harvest",I19=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A19="","",IF(F19=0,"",IF(G19&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D19="Harvest",I19=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -848,7 +848,7 @@
         <v/>
       </c>
       <c r="M20" s="6">
-        <f>IF(A20="","",IF(F20=0,"",IF(G20&lt;0.25,"P0 fix hook",IF(AND(D20="Harvest",I20=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A20="","",IF(F20=0,"",IF(G20&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D20="Harvest",I20=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -862,7 +862,7 @@
         <v/>
       </c>
       <c r="M21" s="6">
-        <f>IF(A21="","",IF(F21=0,"",IF(G21&lt;0.25,"P0 fix hook",IF(AND(D21="Harvest",I21=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A21="","",IF(F21=0,"",IF(G21&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D21="Harvest",I21=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -876,7 +876,7 @@
         <v/>
       </c>
       <c r="M22" s="6">
-        <f>IF(A22="","",IF(F22=0,"",IF(G22&lt;0.25,"P0 fix hook",IF(AND(D22="Harvest",I22=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A22="","",IF(F22=0,"",IF(G22&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D22="Harvest",I22=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -890,7 +890,7 @@
         <v/>
       </c>
       <c r="M23" s="6">
-        <f>IF(A23="","",IF(F23=0,"",IF(G23&lt;0.25,"P0 fix hook",IF(AND(D23="Harvest",I23=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A23="","",IF(F23=0,"",IF(G23&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D23="Harvest",I23=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -904,7 +904,7 @@
         <v/>
       </c>
       <c r="M24" s="6">
-        <f>IF(A24="","",IF(F24=0,"",IF(G24&lt;0.25,"P0 fix hook",IF(AND(D24="Harvest",I24=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A24="","",IF(F24=0,"",IF(G24&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D24="Harvest",I24=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -918,7 +918,7 @@
         <v/>
       </c>
       <c r="M25" s="6">
-        <f>IF(A25="","",IF(F25=0,"",IF(G25&lt;0.25,"P0 fix hook",IF(AND(D25="Harvest",I25=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A25="","",IF(F25=0,"",IF(G25&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D25="Harvest",I25=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -932,7 +932,7 @@
         <v/>
       </c>
       <c r="M26" s="6">
-        <f>IF(A26="","",IF(F26=0,"",IF(G26&lt;0.25,"P0 fix hook",IF(AND(D26="Harvest",I26=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A26="","",IF(F26=0,"",IF(G26&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D26="Harvest",I26=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -946,7 +946,7 @@
         <v/>
       </c>
       <c r="M27" s="6">
-        <f>IF(A27="","",IF(F27=0,"",IF(G27&lt;0.25,"P0 fix hook",IF(AND(D27="Harvest",I27=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A27="","",IF(F27=0,"",IF(G27&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D27="Harvest",I27=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -960,7 +960,7 @@
         <v/>
       </c>
       <c r="M28" s="6">
-        <f>IF(A28="","",IF(F28=0,"",IF(G28&lt;0.25,"P0 fix hook",IF(AND(D28="Harvest",I28=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A28="","",IF(F28=0,"",IF(G28&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D28="Harvest",I28=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v/>
       </c>
       <c r="M29" s="6">
-        <f>IF(A29="","",IF(F29=0,"",IF(G29&lt;0.25,"P0 fix hook",IF(AND(D29="Harvest",I29=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A29="","",IF(F29=0,"",IF(G29&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D29="Harvest",I29=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -988,7 +988,7 @@
         <v/>
       </c>
       <c r="M30" s="6">
-        <f>IF(A30="","",IF(F30=0,"",IF(G30&lt;0.25,"P0 fix hook",IF(AND(D30="Harvest",I30=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A30="","",IF(F30=0,"",IF(G30&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D30="Harvest",I30=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1002,7 +1002,7 @@
         <v/>
       </c>
       <c r="M31" s="6">
-        <f>IF(A31="","",IF(F31=0,"",IF(G31&lt;0.25,"P0 fix hook",IF(AND(D31="Harvest",I31=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A31="","",IF(F31=0,"",IF(G31&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D31="Harvest",I31=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
         <v/>
       </c>
       <c r="M32" s="6">
-        <f>IF(A32="","",IF(F32=0,"",IF(G32&lt;0.25,"P0 fix hook",IF(AND(D32="Harvest",I32=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A32="","",IF(F32=0,"",IF(G32&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D32="Harvest",I32=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
         <v/>
       </c>
       <c r="M33" s="6">
-        <f>IF(A33="","",IF(F33=0,"",IF(G33&lt;0.25,"P0 fix hook",IF(AND(D33="Harvest",I33=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A33="","",IF(F33=0,"",IF(G33&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D33="Harvest",I33=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1044,7 +1044,7 @@
         <v/>
       </c>
       <c r="M34" s="6">
-        <f>IF(A34="","",IF(F34=0,"",IF(G34&lt;0.25,"P0 fix hook",IF(AND(D34="Harvest",I34=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A34="","",IF(F34=0,"",IF(G34&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D34="Harvest",I34=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
         <v/>
       </c>
       <c r="M35" s="6">
-        <f>IF(A35="","",IF(F35=0,"",IF(G35&lt;0.25,"P0 fix hook",IF(AND(D35="Harvest",I35=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A35="","",IF(F35=0,"",IF(G35&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D35="Harvest",I35=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
         <v/>
       </c>
       <c r="M36" s="6">
-        <f>IF(A36="","",IF(F36=0,"",IF(G36&lt;0.25,"P0 fix hook",IF(AND(D36="Harvest",I36=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A36="","",IF(F36=0,"",IF(G36&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D36="Harvest",I36=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
         <v/>
       </c>
       <c r="M37" s="6">
-        <f>IF(A37="","",IF(F37=0,"",IF(G37&lt;0.25,"P0 fix hook",IF(AND(D37="Harvest",I37=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A37="","",IF(F37=0,"",IF(G37&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D37="Harvest",I37=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
         <v/>
       </c>
       <c r="M38" s="6">
-        <f>IF(A38="","",IF(F38=0,"",IF(G38&lt;0.25,"P0 fix hook",IF(AND(D38="Harvest",I38=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A38="","",IF(F38=0,"",IF(G38&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D38="Harvest",I38=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
         <v/>
       </c>
       <c r="M39" s="6">
-        <f>IF(A39="","",IF(F39=0,"",IF(G39&lt;0.25,"P0 fix hook",IF(AND(D39="Harvest",I39=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A39="","",IF(F39=0,"",IF(G39&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D39="Harvest",I39=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
         <v/>
       </c>
       <c r="M40" s="6">
-        <f>IF(A40="","",IF(F40=0,"",IF(G40&lt;0.25,"P0 fix hook",IF(AND(D40="Harvest",I40=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A40="","",IF(F40=0,"",IF(G40&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D40="Harvest",I40=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
         <v/>
       </c>
       <c r="M41" s="6">
-        <f>IF(A41="","",IF(F41=0,"",IF(G41&lt;0.25,"P0 fix hook",IF(AND(D41="Harvest",I41=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A41="","",IF(F41=0,"",IF(G41&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D41="Harvest",I41=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1156,7 +1156,7 @@
         <v/>
       </c>
       <c r="M42" s="6">
-        <f>IF(A42="","",IF(F42=0,"",IF(G42&lt;0.25,"P0 fix hook",IF(AND(D42="Harvest",I42=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A42="","",IF(F42=0,"",IF(G42&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D42="Harvest",I42=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1170,7 +1170,7 @@
         <v/>
       </c>
       <c r="M43" s="6">
-        <f>IF(A43="","",IF(F43=0,"",IF(G43&lt;0.25,"P0 fix hook",IF(AND(D43="Harvest",I43=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A43="","",IF(F43=0,"",IF(G43&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D43="Harvest",I43=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1184,7 +1184,7 @@
         <v/>
       </c>
       <c r="M44" s="6">
-        <f>IF(A44="","",IF(F44=0,"",IF(G44&lt;0.25,"P0 fix hook",IF(AND(D44="Harvest",I44=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A44="","",IF(F44=0,"",IF(G44&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D44="Harvest",I44=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1198,7 +1198,7 @@
         <v/>
       </c>
       <c r="M45" s="6">
-        <f>IF(A45="","",IF(F45=0,"",IF(G45&lt;0.25,"P0 fix hook",IF(AND(D45="Harvest",I45=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A45="","",IF(F45=0,"",IF(G45&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D45="Harvest",I45=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
         <v/>
       </c>
       <c r="M46" s="6">
-        <f>IF(A46="","",IF(F46=0,"",IF(G46&lt;0.25,"P0 fix hook",IF(AND(D46="Harvest",I46=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A46="","",IF(F46=0,"",IF(G46&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D46="Harvest",I46=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
         <v/>
       </c>
       <c r="M47" s="6">
-        <f>IF(A47="","",IF(F47=0,"",IF(G47&lt;0.25,"P0 fix hook",IF(AND(D47="Harvest",I47=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A47="","",IF(F47=0,"",IF(G47&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D47="Harvest",I47=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
         <v/>
       </c>
       <c r="M48" s="6">
-        <f>IF(A48="","",IF(F48=0,"",IF(G48&lt;0.25,"P0 fix hook",IF(AND(D48="Harvest",I48=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A48="","",IF(F48=0,"",IF(G48&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D48="Harvest",I48=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1254,7 +1254,7 @@
         <v/>
       </c>
       <c r="M49" s="6">
-        <f>IF(A49="","",IF(F49=0,"",IF(G49&lt;0.25,"P0 fix hook",IF(AND(D49="Harvest",I49=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A49="","",IF(F49=0,"",IF(G49&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D49="Harvest",I49=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1268,7 +1268,7 @@
         <v/>
       </c>
       <c r="M50" s="6">
-        <f>IF(A50="","",IF(F50=0,"",IF(G50&lt;0.25,"P0 fix hook",IF(AND(D50="Harvest",I50=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A50="","",IF(F50=0,"",IF(G50&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D50="Harvest",I50=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
         <v/>
       </c>
       <c r="M51" s="6">
-        <f>IF(A51="","",IF(F51=0,"",IF(G51&lt;0.25,"P0 fix hook",IF(AND(D51="Harvest",I51=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A51="","",IF(F51=0,"",IF(G51&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D51="Harvest",I51=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1296,7 +1296,7 @@
         <v/>
       </c>
       <c r="M52" s="6">
-        <f>IF(A52="","",IF(F52=0,"",IF(G52&lt;0.25,"P0 fix hook",IF(AND(D52="Harvest",I52=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A52="","",IF(F52=0,"",IF(G52&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D52="Harvest",I52=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
         <v/>
       </c>
       <c r="M53" s="6">
-        <f>IF(A53="","",IF(F53=0,"",IF(G53&lt;0.25,"P0 fix hook",IF(AND(D53="Harvest",I53=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A53="","",IF(F53=0,"",IF(G53&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D53="Harvest",I53=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1324,7 +1324,7 @@
         <v/>
       </c>
       <c r="M54" s="6">
-        <f>IF(A54="","",IF(F54=0,"",IF(G54&lt;0.25,"P0 fix hook",IF(AND(D54="Harvest",I54=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A54="","",IF(F54=0,"",IF(G54&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D54="Harvest",I54=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
         <v/>
       </c>
       <c r="M55" s="6">
-        <f>IF(A55="","",IF(F55=0,"",IF(G55&lt;0.25,"P0 fix hook",IF(AND(D55="Harvest",I55=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A55="","",IF(F55=0,"",IF(G55&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D55="Harvest",I55=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
         <v/>
       </c>
       <c r="M56" s="6">
-        <f>IF(A56="","",IF(F56=0,"",IF(G56&lt;0.25,"P0 fix hook",IF(AND(D56="Harvest",I56=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A56="","",IF(F56=0,"",IF(G56&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D56="Harvest",I56=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1366,7 +1366,7 @@
         <v/>
       </c>
       <c r="M57" s="6">
-        <f>IF(A57="","",IF(F57=0,"",IF(G57&lt;0.25,"P0 fix hook",IF(AND(D57="Harvest",I57=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A57="","",IF(F57=0,"",IF(G57&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D57="Harvest",I57=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1380,7 +1380,7 @@
         <v/>
       </c>
       <c r="M58" s="6">
-        <f>IF(A58="","",IF(F58=0,"",IF(G58&lt;0.25,"P0 fix hook",IF(AND(D58="Harvest",I58=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A58="","",IF(F58=0,"",IF(G58&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D58="Harvest",I58=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
         <v/>
       </c>
       <c r="M59" s="6">
-        <f>IF(A59="","",IF(F59=0,"",IF(G59&lt;0.25,"P0 fix hook",IF(AND(D59="Harvest",I59=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A59="","",IF(F59=0,"",IF(G59&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D59="Harvest",I59=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1408,7 +1408,7 @@
         <v/>
       </c>
       <c r="M60" s="6">
-        <f>IF(A60="","",IF(F60=0,"",IF(G60&lt;0.25,"P0 fix hook",IF(AND(D60="Harvest",I60=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A60="","",IF(F60=0,"",IF(G60&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D60="Harvest",I60=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1422,7 +1422,7 @@
         <v/>
       </c>
       <c r="M61" s="6">
-        <f>IF(A61="","",IF(F61=0,"",IF(G61&lt;0.25,"P0 fix hook",IF(AND(D61="Harvest",I61=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A61="","",IF(F61=0,"",IF(G61&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D61="Harvest",I61=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
         <v/>
       </c>
       <c r="M62" s="6">
-        <f>IF(A62="","",IF(F62=0,"",IF(G62&lt;0.25,"P0 fix hook",IF(AND(D62="Harvest",I62=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A62="","",IF(F62=0,"",IF(G62&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D62="Harvest",I62=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1450,7 +1450,7 @@
         <v/>
       </c>
       <c r="M63" s="6">
-        <f>IF(A63="","",IF(F63=0,"",IF(G63&lt;0.25,"P0 fix hook",IF(AND(D63="Harvest",I63=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A63="","",IF(F63=0,"",IF(G63&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D63="Harvest",I63=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
         <v/>
       </c>
       <c r="M64" s="6">
-        <f>IF(A64="","",IF(F64=0,"",IF(G64&lt;0.25,"P0 fix hook",IF(AND(D64="Harvest",I64=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A64="","",IF(F64=0,"",IF(G64&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D64="Harvest",I64=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
         <v/>
       </c>
       <c r="M65" s="6">
-        <f>IF(A65="","",IF(F65=0,"",IF(G65&lt;0.25,"P0 fix hook",IF(AND(D65="Harvest",I65=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A65="","",IF(F65=0,"",IF(G65&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D65="Harvest",I65=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
         <v/>
       </c>
       <c r="M66" s="6">
-        <f>IF(A66="","",IF(F66=0,"",IF(G66&lt;0.25,"P0 fix hook",IF(AND(D66="Harvest",I66=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A66="","",IF(F66=0,"",IF(G66&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D66="Harvest",I66=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1506,7 +1506,7 @@
         <v/>
       </c>
       <c r="M67" s="6">
-        <f>IF(A67="","",IF(F67=0,"",IF(G67&lt;0.25,"P0 fix hook",IF(AND(D67="Harvest",I67=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A67="","",IF(F67=0,"",IF(G67&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D67="Harvest",I67=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1520,7 +1520,7 @@
         <v/>
       </c>
       <c r="M68" s="6">
-        <f>IF(A68="","",IF(F68=0,"",IF(G68&lt;0.25,"P0 fix hook",IF(AND(D68="Harvest",I68=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A68="","",IF(F68=0,"",IF(G68&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D68="Harvest",I68=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1534,7 +1534,7 @@
         <v/>
       </c>
       <c r="M69" s="6">
-        <f>IF(A69="","",IF(F69=0,"",IF(G69&lt;0.25,"P0 fix hook",IF(AND(D69="Harvest",I69=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A69="","",IF(F69=0,"",IF(G69&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D69="Harvest",I69=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1548,7 +1548,7 @@
         <v/>
       </c>
       <c r="M70" s="6">
-        <f>IF(A70="","",IF(F70=0,"",IF(G70&lt;0.25,"P0 fix hook",IF(AND(D70="Harvest",I70=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A70="","",IF(F70=0,"",IF(G70&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D70="Harvest",I70=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1562,7 +1562,7 @@
         <v/>
       </c>
       <c r="M71" s="6">
-        <f>IF(A71="","",IF(F71=0,"",IF(G71&lt;0.25,"P0 fix hook",IF(AND(D71="Harvest",I71=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A71="","",IF(F71=0,"",IF(G71&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D71="Harvest",I71=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1576,7 +1576,7 @@
         <v/>
       </c>
       <c r="M72" s="6">
-        <f>IF(A72="","",IF(F72=0,"",IF(G72&lt;0.25,"P0 fix hook",IF(AND(D72="Harvest",I72=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A72="","",IF(F72=0,"",IF(G72&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D72="Harvest",I72=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1590,7 +1590,7 @@
         <v/>
       </c>
       <c r="M73" s="6">
-        <f>IF(A73="","",IF(F73=0,"",IF(G73&lt;0.25,"P0 fix hook",IF(AND(D73="Harvest",I73=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A73="","",IF(F73=0,"",IF(G73&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D73="Harvest",I73=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         <v/>
       </c>
       <c r="M74" s="6">
-        <f>IF(A74="","",IF(F74=0,"",IF(G74&lt;0.25,"P0 fix hook",IF(AND(D74="Harvest",I74=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A74="","",IF(F74=0,"",IF(G74&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D74="Harvest",I74=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1618,7 +1618,7 @@
         <v/>
       </c>
       <c r="M75" s="6">
-        <f>IF(A75="","",IF(F75=0,"",IF(G75&lt;0.25,"P0 fix hook",IF(AND(D75="Harvest",I75=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A75="","",IF(F75=0,"",IF(G75&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D75="Harvest",I75=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1632,7 +1632,7 @@
         <v/>
       </c>
       <c r="M76" s="6">
-        <f>IF(A76="","",IF(F76=0,"",IF(G76&lt;0.25,"P0 fix hook",IF(AND(D76="Harvest",I76=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A76="","",IF(F76=0,"",IF(G76&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D76="Harvest",I76=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
         <v/>
       </c>
       <c r="M77" s="6">
-        <f>IF(A77="","",IF(F77=0,"",IF(G77&lt;0.25,"P0 fix hook",IF(AND(D77="Harvest",I77=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A77="","",IF(F77=0,"",IF(G77&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D77="Harvest",I77=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1660,7 +1660,7 @@
         <v/>
       </c>
       <c r="M78" s="6">
-        <f>IF(A78="","",IF(F78=0,"",IF(G78&lt;0.25,"P0 fix hook",IF(AND(D78="Harvest",I78=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A78="","",IF(F78=0,"",IF(G78&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D78="Harvest",I78=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1674,7 +1674,7 @@
         <v/>
       </c>
       <c r="M79" s="6">
-        <f>IF(A79="","",IF(F79=0,"",IF(G79&lt;0.25,"P0 fix hook",IF(AND(D79="Harvest",I79=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A79="","",IF(F79=0,"",IF(G79&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D79="Harvest",I79=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1688,7 +1688,7 @@
         <v/>
       </c>
       <c r="M80" s="6">
-        <f>IF(A80="","",IF(F80=0,"",IF(G80&lt;0.25,"P0 fix hook",IF(AND(D80="Harvest",I80=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A80="","",IF(F80=0,"",IF(G80&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D80="Harvest",I80=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
         <v/>
       </c>
       <c r="M81" s="6">
-        <f>IF(A81="","",IF(F81=0,"",IF(G81&lt;0.25,"P0 fix hook",IF(AND(D81="Harvest",I81=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A81="","",IF(F81=0,"",IF(G81&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D81="Harvest",I81=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1716,7 +1716,7 @@
         <v/>
       </c>
       <c r="M82" s="6">
-        <f>IF(A82="","",IF(F82=0,"",IF(G82&lt;0.25,"P0 fix hook",IF(AND(D82="Harvest",I82=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A82="","",IF(F82=0,"",IF(G82&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D82="Harvest",I82=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
         <v/>
       </c>
       <c r="M83" s="6">
-        <f>IF(A83="","",IF(F83=0,"",IF(G83&lt;0.25,"P0 fix hook",IF(AND(D83="Harvest",I83=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A83="","",IF(F83=0,"",IF(G83&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D83="Harvest",I83=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1744,7 +1744,7 @@
         <v/>
       </c>
       <c r="M84" s="6">
-        <f>IF(A84="","",IF(F84=0,"",IF(G84&lt;0.25,"P0 fix hook",IF(AND(D84="Harvest",I84=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A84="","",IF(F84=0,"",IF(G84&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D84="Harvest",I84=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1758,7 +1758,7 @@
         <v/>
       </c>
       <c r="M85" s="6">
-        <f>IF(A85="","",IF(F85=0,"",IF(G85&lt;0.25,"P0 fix hook",IF(AND(D85="Harvest",I85=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A85="","",IF(F85=0,"",IF(G85&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D85="Harvest",I85=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1772,7 +1772,7 @@
         <v/>
       </c>
       <c r="M86" s="6">
-        <f>IF(A86="","",IF(F86=0,"",IF(G86&lt;0.25,"P0 fix hook",IF(AND(D86="Harvest",I86=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A86="","",IF(F86=0,"",IF(G86&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D86="Harvest",I86=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1786,7 +1786,7 @@
         <v/>
       </c>
       <c r="M87" s="6">
-        <f>IF(A87="","",IF(F87=0,"",IF(G87&lt;0.25,"P0 fix hook",IF(AND(D87="Harvest",I87=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A87="","",IF(F87=0,"",IF(G87&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D87="Harvest",I87=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
         <v/>
       </c>
       <c r="M88" s="6">
-        <f>IF(A88="","",IF(F88=0,"",IF(G88&lt;0.25,"P0 fix hook",IF(AND(D88="Harvest",I88=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A88="","",IF(F88=0,"",IF(G88&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D88="Harvest",I88=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1814,7 +1814,7 @@
         <v/>
       </c>
       <c r="M89" s="6">
-        <f>IF(A89="","",IF(F89=0,"",IF(G89&lt;0.25,"P0 fix hook",IF(AND(D89="Harvest",I89=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A89="","",IF(F89=0,"",IF(G89&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D89="Harvest",I89=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
         <v/>
       </c>
       <c r="M90" s="6">
-        <f>IF(A90="","",IF(F90=0,"",IF(G90&lt;0.25,"P0 fix hook",IF(AND(D90="Harvest",I90=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A90="","",IF(F90=0,"",IF(G90&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D90="Harvest",I90=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1842,7 +1842,7 @@
         <v/>
       </c>
       <c r="M91" s="6">
-        <f>IF(A91="","",IF(F91=0,"",IF(G91&lt;0.25,"P0 fix hook",IF(AND(D91="Harvest",I91=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A91="","",IF(F91=0,"",IF(G91&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D91="Harvest",I91=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
         <v/>
       </c>
       <c r="M92" s="6">
-        <f>IF(A92="","",IF(F92=0,"",IF(G92&lt;0.25,"P0 fix hook",IF(AND(D92="Harvest",I92=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A92="","",IF(F92=0,"",IF(G92&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D92="Harvest",I92=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1870,7 +1870,7 @@
         <v/>
       </c>
       <c r="M93" s="6">
-        <f>IF(A93="","",IF(F93=0,"",IF(G93&lt;0.25,"P0 fix hook",IF(AND(D93="Harvest",I93=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A93="","",IF(F93=0,"",IF(G93&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D93="Harvest",I93=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1884,7 +1884,7 @@
         <v/>
       </c>
       <c r="M94" s="6">
-        <f>IF(A94="","",IF(F94=0,"",IF(G94&lt;0.25,"P0 fix hook",IF(AND(D94="Harvest",I94=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A94="","",IF(F94=0,"",IF(G94&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D94="Harvest",I94=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
         <v/>
       </c>
       <c r="M95" s="6">
-        <f>IF(A95="","",IF(F95=0,"",IF(G95&lt;0.25,"P0 fix hook",IF(AND(D95="Harvest",I95=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A95="","",IF(F95=0,"",IF(G95&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D95="Harvest",I95=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
         <v/>
       </c>
       <c r="M96" s="6">
-        <f>IF(A96="","",IF(F96=0,"",IF(G96&lt;0.25,"P0 fix hook",IF(AND(D96="Harvest",I96=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A96="","",IF(F96=0,"",IF(G96&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D96="Harvest",I96=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1926,7 +1926,7 @@
         <v/>
       </c>
       <c r="M97" s="6">
-        <f>IF(A97="","",IF(F97=0,"",IF(G97&lt;0.25,"P0 fix hook",IF(AND(D97="Harvest",I97=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A97="","",IF(F97=0,"",IF(G97&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D97="Harvest",I97=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1940,7 +1940,7 @@
         <v/>
       </c>
       <c r="M98" s="6">
-        <f>IF(A98="","",IF(F98=0,"",IF(G98&lt;0.25,"P0 fix hook",IF(AND(D98="Harvest",I98=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A98="","",IF(F98=0,"",IF(G98&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D98="Harvest",I98=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1954,7 +1954,7 @@
         <v/>
       </c>
       <c r="M99" s="6">
-        <f>IF(A99="","",IF(F99=0,"",IF(G99&lt;0.25,"P0 fix hook",IF(AND(D99="Harvest",I99=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A99="","",IF(F99=0,"",IF(G99&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D99="Harvest",I99=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
         <v/>
       </c>
       <c r="M100" s="6">
-        <f>IF(A100="","",IF(F100=0,"",IF(G100&lt;0.25,"P0 fix hook",IF(AND(D100="Harvest",I100=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A100="","",IF(F100=0,"",IF(G100&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D100="Harvest",I100=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
         <v/>
       </c>
       <c r="M101" s="6">
-        <f>IF(A101="","",IF(F101=0,"",IF(G101&lt;0.25,"P0 fix hook",IF(AND(D101="Harvest",I101=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A101="","",IF(F101=0,"",IF(G101&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D101="Harvest",I101=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
         <v/>
       </c>
       <c r="M102" s="6">
-        <f>IF(A102="","",IF(F102=0,"",IF(G102&lt;0.25,"P0 fix hook",IF(AND(D102="Harvest",I102=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A102="","",IF(F102=0,"",IF(G102&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D102="Harvest",I102=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2010,7 +2010,7 @@
         <v/>
       </c>
       <c r="M103" s="6">
-        <f>IF(A103="","",IF(F103=0,"",IF(G103&lt;0.25,"P0 fix hook",IF(AND(D103="Harvest",I103=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A103="","",IF(F103=0,"",IF(G103&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D103="Harvest",I103=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2024,7 +2024,7 @@
         <v/>
       </c>
       <c r="M104" s="6">
-        <f>IF(A104="","",IF(F104=0,"",IF(G104&lt;0.25,"P0 fix hook",IF(AND(D104="Harvest",I104=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A104="","",IF(F104=0,"",IF(G104&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D104="Harvest",I104=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2038,7 +2038,7 @@
         <v/>
       </c>
       <c r="M105" s="6">
-        <f>IF(A105="","",IF(F105=0,"",IF(G105&lt;0.25,"P0 fix hook",IF(AND(D105="Harvest",I105=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A105="","",IF(F105=0,"",IF(G105&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D105="Harvest",I105=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
         <v/>
       </c>
       <c r="M106" s="6">
-        <f>IF(A106="","",IF(F106=0,"",IF(G106&lt;0.25,"P0 fix hook",IF(AND(D106="Harvest",I106=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A106="","",IF(F106=0,"",IF(G106&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D106="Harvest",I106=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2066,7 +2066,7 @@
         <v/>
       </c>
       <c r="M107" s="6">
-        <f>IF(A107="","",IF(F107=0,"",IF(G107&lt;0.25,"P0 fix hook",IF(AND(D107="Harvest",I107=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A107="","",IF(F107=0,"",IF(G107&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D107="Harvest",I107=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2080,7 +2080,7 @@
         <v/>
       </c>
       <c r="M108" s="6">
-        <f>IF(A108="","",IF(F108=0,"",IF(G108&lt;0.25,"P0 fix hook",IF(AND(D108="Harvest",I108=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A108="","",IF(F108=0,"",IF(G108&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D108="Harvest",I108=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2094,7 +2094,7 @@
         <v/>
       </c>
       <c r="M109" s="6">
-        <f>IF(A109="","",IF(F109=0,"",IF(G109&lt;0.25,"P0 fix hook",IF(AND(D109="Harvest",I109=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A109="","",IF(F109=0,"",IF(G109&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D109="Harvest",I109=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
         <v/>
       </c>
       <c r="M110" s="6">
-        <f>IF(A110="","",IF(F110=0,"",IF(G110&lt;0.25,"P0 fix hook",IF(AND(D110="Harvest",I110=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A110="","",IF(F110=0,"",IF(G110&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D110="Harvest",I110=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2122,7 +2122,7 @@
         <v/>
       </c>
       <c r="M111" s="6">
-        <f>IF(A111="","",IF(F111=0,"",IF(G111&lt;0.25,"P0 fix hook",IF(AND(D111="Harvest",I111=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A111="","",IF(F111=0,"",IF(G111&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D111="Harvest",I111=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2136,7 +2136,7 @@
         <v/>
       </c>
       <c r="M112" s="6">
-        <f>IF(A112="","",IF(F112=0,"",IF(G112&lt;0.25,"P0 fix hook",IF(AND(D112="Harvest",I112=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A112="","",IF(F112=0,"",IF(G112&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D112="Harvest",I112=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2150,7 +2150,7 @@
         <v/>
       </c>
       <c r="M113" s="6">
-        <f>IF(A113="","",IF(F113=0,"",IF(G113&lt;0.25,"P0 fix hook",IF(AND(D113="Harvest",I113=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A113="","",IF(F113=0,"",IF(G113&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D113="Harvest",I113=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2164,7 +2164,7 @@
         <v/>
       </c>
       <c r="M114" s="6">
-        <f>IF(A114="","",IF(F114=0,"",IF(G114&lt;0.25,"P0 fix hook",IF(AND(D114="Harvest",I114=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A114="","",IF(F114=0,"",IF(G114&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D114="Harvest",I114=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2178,7 +2178,7 @@
         <v/>
       </c>
       <c r="M115" s="6">
-        <f>IF(A115="","",IF(F115=0,"",IF(G115&lt;0.25,"P0 fix hook",IF(AND(D115="Harvest",I115=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A115="","",IF(F115=0,"",IF(G115&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D115="Harvest",I115=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2192,7 +2192,7 @@
         <v/>
       </c>
       <c r="M116" s="6">
-        <f>IF(A116="","",IF(F116=0,"",IF(G116&lt;0.25,"P0 fix hook",IF(AND(D116="Harvest",I116=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A116="","",IF(F116=0,"",IF(G116&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D116="Harvest",I116=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
         <v/>
       </c>
       <c r="M117" s="6">
-        <f>IF(A117="","",IF(F117=0,"",IF(G117&lt;0.25,"P0 fix hook",IF(AND(D117="Harvest",I117=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A117="","",IF(F117=0,"",IF(G117&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D117="Harvest",I117=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2220,7 +2220,7 @@
         <v/>
       </c>
       <c r="M118" s="6">
-        <f>IF(A118="","",IF(F118=0,"",IF(G118&lt;0.25,"P0 fix hook",IF(AND(D118="Harvest",I118=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A118="","",IF(F118=0,"",IF(G118&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D118="Harvest",I118=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="M119" s="6">
-        <f>IF(A119="","",IF(F119=0,"",IF(G119&lt;0.25,"P0 fix hook",IF(AND(D119="Harvest",I119=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A119="","",IF(F119=0,"",IF(G119&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D119="Harvest",I119=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2248,7 +2248,7 @@
         <v/>
       </c>
       <c r="M120" s="6">
-        <f>IF(A120="","",IF(F120=0,"",IF(G120&lt;0.25,"P0 fix hook",IF(AND(D120="Harvest",I120=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A120="","",IF(F120=0,"",IF(G120&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D120="Harvest",I120=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2262,7 +2262,7 @@
         <v/>
       </c>
       <c r="M121" s="6">
-        <f>IF(A121="","",IF(F121=0,"",IF(G121&lt;0.25,"P0 fix hook",IF(AND(D121="Harvest",I121=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A121="","",IF(F121=0,"",IF(G121&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D121="Harvest",I121=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2276,7 +2276,7 @@
         <v/>
       </c>
       <c r="M122" s="6">
-        <f>IF(A122="","",IF(F122=0,"",IF(G122&lt;0.25,"P0 fix hook",IF(AND(D122="Harvest",I122=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A122="","",IF(F122=0,"",IF(G122&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D122="Harvest",I122=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2290,7 +2290,7 @@
         <v/>
       </c>
       <c r="M123" s="6">
-        <f>IF(A123="","",IF(F123=0,"",IF(G123&lt;0.25,"P0 fix hook",IF(AND(D123="Harvest",I123=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A123="","",IF(F123=0,"",IF(G123&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D123="Harvest",I123=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2304,7 +2304,7 @@
         <v/>
       </c>
       <c r="M124" s="6">
-        <f>IF(A124="","",IF(F124=0,"",IF(G124&lt;0.25,"P0 fix hook",IF(AND(D124="Harvest",I124=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A124="","",IF(F124=0,"",IF(G124&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D124="Harvest",I124=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2318,7 +2318,7 @@
         <v/>
       </c>
       <c r="M125" s="6">
-        <f>IF(A125="","",IF(F125=0,"",IF(G125&lt;0.25,"P0 fix hook",IF(AND(D125="Harvest",I125=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A125="","",IF(F125=0,"",IF(G125&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D125="Harvest",I125=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2332,7 +2332,7 @@
         <v/>
       </c>
       <c r="M126" s="6">
-        <f>IF(A126="","",IF(F126=0,"",IF(G126&lt;0.25,"P0 fix hook",IF(AND(D126="Harvest",I126=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A126="","",IF(F126=0,"",IF(G126&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D126="Harvest",I126=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2346,7 +2346,7 @@
         <v/>
       </c>
       <c r="M127" s="6">
-        <f>IF(A127="","",IF(F127=0,"",IF(G127&lt;0.25,"P0 fix hook",IF(AND(D127="Harvest",I127=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A127="","",IF(F127=0,"",IF(G127&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D127="Harvest",I127=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
         <v/>
       </c>
       <c r="M128" s="6">
-        <f>IF(A128="","",IF(F128=0,"",IF(G128&lt;0.25,"P0 fix hook",IF(AND(D128="Harvest",I128=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A128="","",IF(F128=0,"",IF(G128&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D128="Harvest",I128=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2374,7 +2374,7 @@
         <v/>
       </c>
       <c r="M129" s="6">
-        <f>IF(A129="","",IF(F129=0,"",IF(G129&lt;0.25,"P0 fix hook",IF(AND(D129="Harvest",I129=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A129="","",IF(F129=0,"",IF(G129&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D129="Harvest",I129=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2388,7 +2388,7 @@
         <v/>
       </c>
       <c r="M130" s="6">
-        <f>IF(A130="","",IF(F130=0,"",IF(G130&lt;0.25,"P0 fix hook",IF(AND(D130="Harvest",I130=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A130="","",IF(F130=0,"",IF(G130&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D130="Harvest",I130=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2402,7 +2402,7 @@
         <v/>
       </c>
       <c r="M131" s="6">
-        <f>IF(A131="","",IF(F131=0,"",IF(G131&lt;0.25,"P0 fix hook",IF(AND(D131="Harvest",I131=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A131="","",IF(F131=0,"",IF(G131&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D131="Harvest",I131=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2416,7 +2416,7 @@
         <v/>
       </c>
       <c r="M132" s="6">
-        <f>IF(A132="","",IF(F132=0,"",IF(G132&lt;0.25,"P0 fix hook",IF(AND(D132="Harvest",I132=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A132="","",IF(F132=0,"",IF(G132&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D132="Harvest",I132=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2430,7 +2430,7 @@
         <v/>
       </c>
       <c r="M133" s="6">
-        <f>IF(A133="","",IF(F133=0,"",IF(G133&lt;0.25,"P0 fix hook",IF(AND(D133="Harvest",I133=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A133="","",IF(F133=0,"",IF(G133&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D133="Harvest",I133=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2444,7 +2444,7 @@
         <v/>
       </c>
       <c r="M134" s="6">
-        <f>IF(A134="","",IF(F134=0,"",IF(G134&lt;0.25,"P0 fix hook",IF(AND(D134="Harvest",I134=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A134="","",IF(F134=0,"",IF(G134&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D134="Harvest",I134=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2458,7 +2458,7 @@
         <v/>
       </c>
       <c r="M135" s="6">
-        <f>IF(A135="","",IF(F135=0,"",IF(G135&lt;0.25,"P0 fix hook",IF(AND(D135="Harvest",I135=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A135="","",IF(F135=0,"",IF(G135&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D135="Harvest",I135=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2472,7 +2472,7 @@
         <v/>
       </c>
       <c r="M136" s="6">
-        <f>IF(A136="","",IF(F136=0,"",IF(G136&lt;0.25,"P0 fix hook",IF(AND(D136="Harvest",I136=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A136="","",IF(F136=0,"",IF(G136&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D136="Harvest",I136=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
         <v/>
       </c>
       <c r="M137" s="6">
-        <f>IF(A137="","",IF(F137=0,"",IF(G137&lt;0.25,"P0 fix hook",IF(AND(D137="Harvest",I137=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A137="","",IF(F137=0,"",IF(G137&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D137="Harvest",I137=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2500,7 +2500,7 @@
         <v/>
       </c>
       <c r="M138" s="6">
-        <f>IF(A138="","",IF(F138=0,"",IF(G138&lt;0.25,"P0 fix hook",IF(AND(D138="Harvest",I138=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A138="","",IF(F138=0,"",IF(G138&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D138="Harvest",I138=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2514,7 +2514,7 @@
         <v/>
       </c>
       <c r="M139" s="6">
-        <f>IF(A139="","",IF(F139=0,"",IF(G139&lt;0.25,"P0 fix hook",IF(AND(D139="Harvest",I139=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A139="","",IF(F139=0,"",IF(G139&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D139="Harvest",I139=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2528,7 +2528,7 @@
         <v/>
       </c>
       <c r="M140" s="6">
-        <f>IF(A140="","",IF(F140=0,"",IF(G140&lt;0.25,"P0 fix hook",IF(AND(D140="Harvest",I140=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A140="","",IF(F140=0,"",IF(G140&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D140="Harvest",I140=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2542,7 +2542,7 @@
         <v/>
       </c>
       <c r="M141" s="6">
-        <f>IF(A141="","",IF(F141=0,"",IF(G141&lt;0.25,"P0 fix hook",IF(AND(D141="Harvest",I141=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A141="","",IF(F141=0,"",IF(G141&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D141="Harvest",I141=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2556,7 +2556,7 @@
         <v/>
       </c>
       <c r="M142" s="6">
-        <f>IF(A142="","",IF(F142=0,"",IF(G142&lt;0.25,"P0 fix hook",IF(AND(D142="Harvest",I142=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A142="","",IF(F142=0,"",IF(G142&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D142="Harvest",I142=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2570,7 +2570,7 @@
         <v/>
       </c>
       <c r="M143" s="6">
-        <f>IF(A143="","",IF(F143=0,"",IF(G143&lt;0.25,"P0 fix hook",IF(AND(D143="Harvest",I143=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A143="","",IF(F143=0,"",IF(G143&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D143="Harvest",I143=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2584,7 +2584,7 @@
         <v/>
       </c>
       <c r="M144" s="6">
-        <f>IF(A144="","",IF(F144=0,"",IF(G144&lt;0.25,"P0 fix hook",IF(AND(D144="Harvest",I144=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A144="","",IF(F144=0,"",IF(G144&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D144="Harvest",I144=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2598,7 +2598,7 @@
         <v/>
       </c>
       <c r="M145" s="6">
-        <f>IF(A145="","",IF(F145=0,"",IF(G145&lt;0.25,"P0 fix hook",IF(AND(D145="Harvest",I145=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A145="","",IF(F145=0,"",IF(G145&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D145="Harvest",I145=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v/>
       </c>
       <c r="M146" s="6">
-        <f>IF(A146="","",IF(F146=0,"",IF(G146&lt;0.25,"P0 fix hook",IF(AND(D146="Harvest",I146=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A146="","",IF(F146=0,"",IF(G146&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D146="Harvest",I146=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2626,7 +2626,7 @@
         <v/>
       </c>
       <c r="M147" s="6">
-        <f>IF(A147="","",IF(F147=0,"",IF(G147&lt;0.25,"P0 fix hook",IF(AND(D147="Harvest",I147=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A147="","",IF(F147=0,"",IF(G147&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D147="Harvest",I147=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2640,7 +2640,7 @@
         <v/>
       </c>
       <c r="M148" s="6">
-        <f>IF(A148="","",IF(F148=0,"",IF(G148&lt;0.25,"P0 fix hook",IF(AND(D148="Harvest",I148=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A148="","",IF(F148=0,"",IF(G148&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D148="Harvest",I148=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2654,7 +2654,7 @@
         <v/>
       </c>
       <c r="M149" s="6">
-        <f>IF(A149="","",IF(F149=0,"",IF(G149&lt;0.25,"P0 fix hook",IF(AND(D149="Harvest",I149=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A149="","",IF(F149=0,"",IF(G149&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D149="Harvest",I149=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2668,7 +2668,7 @@
         <v/>
       </c>
       <c r="M150" s="6">
-        <f>IF(A150="","",IF(F150=0,"",IF(G150&lt;0.25,"P0 fix hook",IF(AND(D150="Harvest",I150=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A150="","",IF(F150=0,"",IF(G150&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D150="Harvest",I150=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2682,7 +2682,7 @@
         <v/>
       </c>
       <c r="M151" s="6">
-        <f>IF(A151="","",IF(F151=0,"",IF(G151&lt;0.25,"P0 fix hook",IF(AND(D151="Harvest",I151=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A151="","",IF(F151=0,"",IF(G151&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D151="Harvest",I151=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2696,7 +2696,7 @@
         <v/>
       </c>
       <c r="M152" s="6">
-        <f>IF(A152="","",IF(F152=0,"",IF(G152&lt;0.25,"P0 fix hook",IF(AND(D152="Harvest",I152=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A152="","",IF(F152=0,"",IF(G152&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D152="Harvest",I152=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2710,7 +2710,7 @@
         <v/>
       </c>
       <c r="M153" s="6">
-        <f>IF(A153="","",IF(F153=0,"",IF(G153&lt;0.25,"P0 fix hook",IF(AND(D153="Harvest",I153=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A153="","",IF(F153=0,"",IF(G153&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D153="Harvest",I153=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2724,7 +2724,7 @@
         <v/>
       </c>
       <c r="M154" s="6">
-        <f>IF(A154="","",IF(F154=0,"",IF(G154&lt;0.25,"P0 fix hook",IF(AND(D154="Harvest",I154=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A154="","",IF(F154=0,"",IF(G154&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D154="Harvest",I154=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v/>
       </c>
       <c r="M155" s="6">
-        <f>IF(A155="","",IF(F155=0,"",IF(G155&lt;0.25,"P0 fix hook",IF(AND(D155="Harvest",I155=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A155="","",IF(F155=0,"",IF(G155&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D155="Harvest",I155=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2752,7 +2752,7 @@
         <v/>
       </c>
       <c r="M156" s="6">
-        <f>IF(A156="","",IF(F156=0,"",IF(G156&lt;0.25,"P0 fix hook",IF(AND(D156="Harvest",I156=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A156="","",IF(F156=0,"",IF(G156&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D156="Harvest",I156=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2766,7 +2766,7 @@
         <v/>
       </c>
       <c r="M157" s="6">
-        <f>IF(A157="","",IF(F157=0,"",IF(G157&lt;0.25,"P0 fix hook",IF(AND(D157="Harvest",I157=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A157="","",IF(F157=0,"",IF(G157&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D157="Harvest",I157=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2780,7 +2780,7 @@
         <v/>
       </c>
       <c r="M158" s="6">
-        <f>IF(A158="","",IF(F158=0,"",IF(G158&lt;0.25,"P0 fix hook",IF(AND(D158="Harvest",I158=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A158="","",IF(F158=0,"",IF(G158&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D158="Harvest",I158=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2794,7 +2794,7 @@
         <v/>
       </c>
       <c r="M159" s="6">
-        <f>IF(A159="","",IF(F159=0,"",IF(G159&lt;0.25,"P0 fix hook",IF(AND(D159="Harvest",I159=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A159="","",IF(F159=0,"",IF(G159&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D159="Harvest",I159=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2808,7 +2808,7 @@
         <v/>
       </c>
       <c r="M160" s="6">
-        <f>IF(A160="","",IF(F160=0,"",IF(G160&lt;0.25,"P0 fix hook",IF(AND(D160="Harvest",I160=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A160="","",IF(F160=0,"",IF(G160&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D160="Harvest",I160=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2822,7 +2822,7 @@
         <v/>
       </c>
       <c r="M161" s="6">
-        <f>IF(A161="","",IF(F161=0,"",IF(G161&lt;0.25,"P0 fix hook",IF(AND(D161="Harvest",I161=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A161="","",IF(F161=0,"",IF(G161&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D161="Harvest",I161=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2836,7 +2836,7 @@
         <v/>
       </c>
       <c r="M162" s="6">
-        <f>IF(A162="","",IF(F162=0,"",IF(G162&lt;0.25,"P0 fix hook",IF(AND(D162="Harvest",I162=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A162="","",IF(F162=0,"",IF(G162&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D162="Harvest",I162=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
         <v/>
       </c>
       <c r="M163" s="6">
-        <f>IF(A163="","",IF(F163=0,"",IF(G163&lt;0.25,"P0 fix hook",IF(AND(D163="Harvest",I163=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A163="","",IF(F163=0,"",IF(G163&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D163="Harvest",I163=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
         <v/>
       </c>
       <c r="M164" s="6">
-        <f>IF(A164="","",IF(F164=0,"",IF(G164&lt;0.25,"P0 fix hook",IF(AND(D164="Harvest",I164=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A164="","",IF(F164=0,"",IF(G164&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D164="Harvest",I164=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2878,7 +2878,7 @@
         <v/>
       </c>
       <c r="M165" s="6">
-        <f>IF(A165="","",IF(F165=0,"",IF(G165&lt;0.25,"P0 fix hook",IF(AND(D165="Harvest",I165=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A165="","",IF(F165=0,"",IF(G165&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D165="Harvest",I165=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2892,7 +2892,7 @@
         <v/>
       </c>
       <c r="M166" s="6">
-        <f>IF(A166="","",IF(F166=0,"",IF(G166&lt;0.25,"P0 fix hook",IF(AND(D166="Harvest",I166=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A166="","",IF(F166=0,"",IF(G166&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D166="Harvest",I166=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2906,7 +2906,7 @@
         <v/>
       </c>
       <c r="M167" s="6">
-        <f>IF(A167="","",IF(F167=0,"",IF(G167&lt;0.25,"P0 fix hook",IF(AND(D167="Harvest",I167=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A167="","",IF(F167=0,"",IF(G167&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D167="Harvest",I167=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2920,7 +2920,7 @@
         <v/>
       </c>
       <c r="M168" s="6">
-        <f>IF(A168="","",IF(F168=0,"",IF(G168&lt;0.25,"P0 fix hook",IF(AND(D168="Harvest",I168=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A168="","",IF(F168=0,"",IF(G168&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D168="Harvest",I168=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2934,7 +2934,7 @@
         <v/>
       </c>
       <c r="M169" s="6">
-        <f>IF(A169="","",IF(F169=0,"",IF(G169&lt;0.25,"P0 fix hook",IF(AND(D169="Harvest",I169=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A169="","",IF(F169=0,"",IF(G169&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D169="Harvest",I169=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2948,7 +2948,7 @@
         <v/>
       </c>
       <c r="M170" s="6">
-        <f>IF(A170="","",IF(F170=0,"",IF(G170&lt;0.25,"P0 fix hook",IF(AND(D170="Harvest",I170=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A170="","",IF(F170=0,"",IF(G170&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D170="Harvest",I170=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2962,7 +2962,7 @@
         <v/>
       </c>
       <c r="M171" s="6">
-        <f>IF(A171="","",IF(F171=0,"",IF(G171&lt;0.25,"P0 fix hook",IF(AND(D171="Harvest",I171=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A171="","",IF(F171=0,"",IF(G171&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D171="Harvest",I171=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
         <v/>
       </c>
       <c r="M172" s="6">
-        <f>IF(A172="","",IF(F172=0,"",IF(G172&lt;0.25,"P0 fix hook",IF(AND(D172="Harvest",I172=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A172="","",IF(F172=0,"",IF(G172&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D172="Harvest",I172=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
         <v/>
       </c>
       <c r="M173" s="6">
-        <f>IF(A173="","",IF(F173=0,"",IF(G173&lt;0.25,"P0 fix hook",IF(AND(D173="Harvest",I173=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A173="","",IF(F173=0,"",IF(G173&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D173="Harvest",I173=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3004,7 +3004,7 @@
         <v/>
       </c>
       <c r="M174" s="6">
-        <f>IF(A174="","",IF(F174=0,"",IF(G174&lt;0.25,"P0 fix hook",IF(AND(D174="Harvest",I174=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A174="","",IF(F174=0,"",IF(G174&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D174="Harvest",I174=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3018,7 +3018,7 @@
         <v/>
       </c>
       <c r="M175" s="6">
-        <f>IF(A175="","",IF(F175=0,"",IF(G175&lt;0.25,"P0 fix hook",IF(AND(D175="Harvest",I175=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A175="","",IF(F175=0,"",IF(G175&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D175="Harvest",I175=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3032,7 +3032,7 @@
         <v/>
       </c>
       <c r="M176" s="6">
-        <f>IF(A176="","",IF(F176=0,"",IF(G176&lt;0.25,"P0 fix hook",IF(AND(D176="Harvest",I176=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A176="","",IF(F176=0,"",IF(G176&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D176="Harvest",I176=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3046,7 +3046,7 @@
         <v/>
       </c>
       <c r="M177" s="6">
-        <f>IF(A177="","",IF(F177=0,"",IF(G177&lt;0.25,"P0 fix hook",IF(AND(D177="Harvest",I177=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A177="","",IF(F177=0,"",IF(G177&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D177="Harvest",I177=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3060,7 +3060,7 @@
         <v/>
       </c>
       <c r="M178" s="6">
-        <f>IF(A178="","",IF(F178=0,"",IF(G178&lt;0.25,"P0 fix hook",IF(AND(D178="Harvest",I178=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A178="","",IF(F178=0,"",IF(G178&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D178="Harvest",I178=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3074,7 +3074,7 @@
         <v/>
       </c>
       <c r="M179" s="6">
-        <f>IF(A179="","",IF(F179=0,"",IF(G179&lt;0.25,"P0 fix hook",IF(AND(D179="Harvest",I179=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A179="","",IF(F179=0,"",IF(G179&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D179="Harvest",I179=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3088,7 +3088,7 @@
         <v/>
       </c>
       <c r="M180" s="6">
-        <f>IF(A180="","",IF(F180=0,"",IF(G180&lt;0.25,"P0 fix hook",IF(AND(D180="Harvest",I180=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A180="","",IF(F180=0,"",IF(G180&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D180="Harvest",I180=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3102,7 +3102,7 @@
         <v/>
       </c>
       <c r="M181" s="6">
-        <f>IF(A181="","",IF(F181=0,"",IF(G181&lt;0.25,"P0 fix hook",IF(AND(D181="Harvest",I181=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A181="","",IF(F181=0,"",IF(G181&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D181="Harvest",I181=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
         <v/>
       </c>
       <c r="M182" s="6">
-        <f>IF(A182="","",IF(F182=0,"",IF(G182&lt;0.25,"P0 fix hook",IF(AND(D182="Harvest",I182=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A182="","",IF(F182=0,"",IF(G182&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D182="Harvest",I182=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3130,7 +3130,7 @@
         <v/>
       </c>
       <c r="M183" s="6">
-        <f>IF(A183="","",IF(F183=0,"",IF(G183&lt;0.25,"P0 fix hook",IF(AND(D183="Harvest",I183=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A183="","",IF(F183=0,"",IF(G183&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D183="Harvest",I183=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3144,7 +3144,7 @@
         <v/>
       </c>
       <c r="M184" s="6">
-        <f>IF(A184="","",IF(F184=0,"",IF(G184&lt;0.25,"P0 fix hook",IF(AND(D184="Harvest",I184=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A184="","",IF(F184=0,"",IF(G184&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D184="Harvest",I184=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
         <v/>
       </c>
       <c r="M185" s="6">
-        <f>IF(A185="","",IF(F185=0,"",IF(G185&lt;0.25,"P0 fix hook",IF(AND(D185="Harvest",I185=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A185="","",IF(F185=0,"",IF(G185&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D185="Harvest",I185=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3172,7 +3172,7 @@
         <v/>
       </c>
       <c r="M186" s="6">
-        <f>IF(A186="","",IF(F186=0,"",IF(G186&lt;0.25,"P0 fix hook",IF(AND(D186="Harvest",I186=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A186="","",IF(F186=0,"",IF(G186&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D186="Harvest",I186=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3186,7 +3186,7 @@
         <v/>
       </c>
       <c r="M187" s="6">
-        <f>IF(A187="","",IF(F187=0,"",IF(G187&lt;0.25,"P0 fix hook",IF(AND(D187="Harvest",I187=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A187="","",IF(F187=0,"",IF(G187&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D187="Harvest",I187=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3200,7 +3200,7 @@
         <v/>
       </c>
       <c r="M188" s="6">
-        <f>IF(A188="","",IF(F188=0,"",IF(G188&lt;0.25,"P0 fix hook",IF(AND(D188="Harvest",I188=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A188="","",IF(F188=0,"",IF(G188&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D188="Harvest",I188=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3214,7 +3214,7 @@
         <v/>
       </c>
       <c r="M189" s="6">
-        <f>IF(A189="","",IF(F189=0,"",IF(G189&lt;0.25,"P0 fix hook",IF(AND(D189="Harvest",I189=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A189="","",IF(F189=0,"",IF(G189&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D189="Harvest",I189=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3228,7 +3228,7 @@
         <v/>
       </c>
       <c r="M190" s="6">
-        <f>IF(A190="","",IF(F190=0,"",IF(G190&lt;0.25,"P0 fix hook",IF(AND(D190="Harvest",I190=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A190="","",IF(F190=0,"",IF(G190&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D190="Harvest",I190=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v/>
       </c>
       <c r="M191" s="6">
-        <f>IF(A191="","",IF(F191=0,"",IF(G191&lt;0.25,"P0 fix hook",IF(AND(D191="Harvest",I191=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A191="","",IF(F191=0,"",IF(G191&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D191="Harvest",I191=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3256,7 +3256,7 @@
         <v/>
       </c>
       <c r="M192" s="6">
-        <f>IF(A192="","",IF(F192=0,"",IF(G192&lt;0.25,"P0 fix hook",IF(AND(D192="Harvest",I192=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A192="","",IF(F192=0,"",IF(G192&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D192="Harvest",I192=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3270,7 +3270,7 @@
         <v/>
       </c>
       <c r="M193" s="6">
-        <f>IF(A193="","",IF(F193=0,"",IF(G193&lt;0.25,"P0 fix hook",IF(AND(D193="Harvest",I193=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A193="","",IF(F193=0,"",IF(G193&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D193="Harvest",I193=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3284,7 +3284,7 @@
         <v/>
       </c>
       <c r="M194" s="6">
-        <f>IF(A194="","",IF(F194=0,"",IF(G194&lt;0.25,"P0 fix hook",IF(AND(D194="Harvest",I194=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A194="","",IF(F194=0,"",IF(G194&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D194="Harvest",I194=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
         <v/>
       </c>
       <c r="M195" s="6">
-        <f>IF(A195="","",IF(F195=0,"",IF(G195&lt;0.25,"P0 fix hook",IF(AND(D195="Harvest",I195=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A195="","",IF(F195=0,"",IF(G195&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D195="Harvest",I195=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3312,7 +3312,7 @@
         <v/>
       </c>
       <c r="M196" s="6">
-        <f>IF(A196="","",IF(F196=0,"",IF(G196&lt;0.25,"P0 fix hook",IF(AND(D196="Harvest",I196=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A196="","",IF(F196=0,"",IF(G196&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D196="Harvest",I196=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3326,7 +3326,7 @@
         <v/>
       </c>
       <c r="M197" s="6">
-        <f>IF(A197="","",IF(F197=0,"",IF(G197&lt;0.25,"P0 fix hook",IF(AND(D197="Harvest",I197=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A197="","",IF(F197=0,"",IF(G197&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D197="Harvest",I197=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3340,7 +3340,7 @@
         <v/>
       </c>
       <c r="M198" s="6">
-        <f>IF(A198="","",IF(F198=0,"",IF(G198&lt;0.25,"P0 fix hook",IF(AND(D198="Harvest",I198=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A198="","",IF(F198=0,"",IF(G198&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D198="Harvest",I198=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
         <v/>
       </c>
       <c r="M199" s="6">
-        <f>IF(A199="","",IF(F199=0,"",IF(G199&lt;0.25,"P0 fix hook",IF(AND(D199="Harvest",I199=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A199="","",IF(F199=0,"",IF(G199&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D199="Harvest",I199=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
         <v/>
       </c>
       <c r="M200" s="6">
-        <f>IF(A200="","",IF(F200=0,"",IF(G200&lt;0.25,"P0 fix hook",IF(AND(D200="Harvest",I200=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A200="","",IF(F200=0,"",IF(G200&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D200="Harvest",I200=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3382,7 +3382,7 @@
         <v/>
       </c>
       <c r="M201" s="6">
-        <f>IF(A201="","",IF(F201=0,"",IF(G201&lt;0.25,"P0 fix hook",IF(AND(D201="Harvest",I201=0),"P1 check proof/CTA","P2 keep"))))</f>
+        <f>IF(A201="","",IF(F201=0,"",IF(G201&lt;0.6,"P0 fix hook (6s retention under 60%)",IF(AND(D201="Harvest",I201=0),"P1 check proof/CTA","P2 keep"))))</f>
         <v/>
       </c>
     </row>
@@ -3441,7 +3441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Log every published asset, good or bad. Triage P0 (fix opening now) / P1 (watch) / P2 (leave).</t>
+          <t>Log every published asset, good or bad. Triage P0 (fix opening now) / P1 (watch) / P2 (leave). Triage gate: CC's first-6-second rule (≈60 of 100 viewers through second 6 earns the next traffic pool).</t>
         </is>
       </c>
     </row>

</xml_diff>